<commit_message>
docs: sync references and sealed progress
</commit_message>
<xml_diff>
--- a/docs/reference/00.Project-Progress-Control｜Pickleball Booking Platform.xlsx
+++ b/docs/reference/00.Project-Progress-Control｜Pickleball Booking Platform.xlsx
@@ -14,386 +14,398 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="151">
   <si>
     <t>Pickleball Booking Platform｜專案進度控管總覽</t>
   </si>
   <si>
-    <t>最後更新：2026-08-12 14:49｜目前階段：Phase 10 — Development｜10 Review Gate PASS｜目前接續：10.1 Repository Bootstrap</t>
+    <t>最後更新：2026-08-17 22:46｜目前階段：Phase 10 — Development｜Slice 1 Merge Gate PASS / Closed｜目前接續：Slice 2 — Coach Supply + Lesson Demand</t>
   </si>
   <si>
     <t>整體成熟度</t>
   </si>
   <si>
-    <t>Implementation Ready</t>
-  </si>
-  <si>
-    <t>01～10 Approved Baseline 已完成；10 Development Master Plan / Repository / Vertical Slice / Test / CI / Security 開發基線已通過 Review Gate</t>
+    <t>Implementation In Progress</t>
+  </si>
+  <si>
+    <t>01～10 Approved Baseline 已完成；Slice 0 Engineering Foundation 與 Slice 1 Identity / LINE Login / Me / RBAC + Organization Scope 已完成、PR #1 已 Merge、遠端 CI 全綠。</t>
   </si>
   <si>
     <t>推薦接續方向
-P0：10.1 Repository Bootstrap
-10 Development Review Gate 已通過；下一步建立實際 Monorepo、Backend / Frontend、PostgreSQL 18、Flyway、Testcontainers 與 CI skeleton。後續實作若發現規格缺口，以 forward-fix 回補 04～10 Source of Truth。</t>
+P0：Slice 2 — Coach Supply + Lesson Demand
+以已完成的 Identity / RBAC / Organization Scope 為基礎，實作 Coach Application / Availability 與 Student Lesson Request 的建立、送審、審核、Authorization、Idempotency、OpenAPI、Frontend 與測試。</t>
   </si>
   <si>
     <t>Development Ready 模組</t>
   </si>
   <si>
+    <t>Slice 0–1 Closed</t>
+  </si>
+  <si>
+    <t>Repository Bootstrap / Engineering Foundation 與 Slice 1 已完成本機驗收、PR、Merge Gate 與 GitHub Actions；main 已同步。</t>
+  </si>
+  <si>
+    <t>優先接續單元</t>
+  </si>
+  <si>
+    <t>Slice 2 — Coach Supply + Lesson Demand</t>
+  </si>
+  <si>
+    <t>下一個正式 Vertical Slice：Coach Application / Availability + Student Lesson Request；延續 OpenAPI 單一來源、PostgreSQL Testcontainers、Security / Organization Scope 與 P0 E2E Gate。</t>
+  </si>
+  <si>
+    <t>主要風險</t>
+  </si>
+  <si>
+    <t>Slice 2 狀態轉換 / Organization Scope / Idempotency</t>
+  </si>
+  <si>
+    <t>Slice 2 會首次大量使用 Coach 與 Student 的資源級授權與 DRAFT → SUBMITTED / approval 狀態轉換；需維持 Backend 為最終授權邊界並以 DB constraint + integration test 保護一致性。</t>
+  </si>
+  <si>
+    <t>階段</t>
+  </si>
+  <si>
+    <t>狀態</t>
+  </si>
+  <si>
+    <t>成熟度</t>
+  </si>
+  <si>
+    <t>下一步</t>
+  </si>
+  <si>
+    <t>00 Project Definition</t>
+  </si>
+  <si>
+    <t>🟢 Done</t>
+  </si>
+  <si>
+    <t>高</t>
+  </si>
+  <si>
+    <t>已完成，維護即可</t>
+  </si>
+  <si>
+    <t>優先級</t>
+  </si>
+  <si>
+    <t>模組</t>
+  </si>
+  <si>
+    <t>符號</t>
+  </si>
+  <si>
+    <t>01 PRD</t>
+  </si>
+  <si>
+    <t>PRD 已確認，作為 MVP 需求基準</t>
+  </si>
+  <si>
+    <t>02 Business Rules</t>
+  </si>
+  <si>
+    <t>Design Baseline，作為 DB / API / Domain / Test 依據</t>
+  </si>
+  <si>
+    <t>03 System Architecture</t>
+  </si>
+  <si>
+    <t>架構基線完成，可支撐 04 Database Design</t>
+  </si>
+  <si>
+    <t>04 Database Design</t>
+  </si>
+  <si>
+    <t>已通過 04-1～04-6 Review Gate，作為 05 輸入基線</t>
+  </si>
+  <si>
+    <t>05 Domain Model</t>
+  </si>
+  <si>
+    <t>Business Rule</t>
+  </si>
+  <si>
+    <t>Review Gate PASS，可作為 06 API Specification 輸入基線</t>
+  </si>
+  <si>
+    <t>單元</t>
+  </si>
+  <si>
+    <t>06 API Specification</t>
+  </si>
+  <si>
+    <t>說明</t>
+  </si>
+  <si>
+    <t>DB</t>
+  </si>
+  <si>
+    <t>Review Gate PASS；含 Permission / Security、Idempotency、Reschedule、Pricing、Refund</t>
+  </si>
+  <si>
+    <t>要完成的事情</t>
+  </si>
+  <si>
+    <t>07 UI/UX Flow</t>
+  </si>
+  <si>
+    <t>Domain Model</t>
+  </si>
+  <si>
+    <t>07 Review Gate PASS / Approved Baseline</t>
+  </si>
+  <si>
+    <t>完成條件</t>
+  </si>
+  <si>
+    <t>08 Test Strategy</t>
+  </si>
+  <si>
+    <t>08 Review Gate PASS / Approved Baseline；Test Strategy 基線已確認</t>
+  </si>
+  <si>
+    <t>Permission</t>
+  </si>
+  <si>
+    <t>09 Deployment / DevOps</t>
+  </si>
+  <si>
+    <t>建議接續順序</t>
+  </si>
+  <si>
+    <t>09 Review Gate PASS / Approved Baseline；GCP-first Deployment / DevOps 基線已確認</t>
+  </si>
+  <si>
+    <t>API</t>
+  </si>
+  <si>
+    <t>🟢</t>
+  </si>
+  <si>
+    <t>10 Development</t>
+  </si>
+  <si>
+    <t>🟡 In Progress</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>11 Future Extensions</t>
+  </si>
+  <si>
     <t>Ready</t>
   </si>
   <si>
-    <t>01～10 Design + Development Plan Baseline 已完成；P0 模組可正式進入 Repository Bootstrap 與 Vertical Slice Coding</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>優先接續單元</t>
-  </si>
-  <si>
-    <t>10.1 Repository Bootstrap</t>
-  </si>
-  <si>
-    <t>建立 Monorepo、Spring Boot / Maven Wrapper、React workspaces、PostgreSQL 18 local stack、Flyway baseline、Testcontainers 與 GitHub Actions CI skeleton</t>
-  </si>
-  <si>
-    <t>主要風險</t>
-  </si>
-  <si>
-    <t>UI / API 狀態與權限一致性</t>
-  </si>
-  <si>
-    <t>避免畫面提供後端不允許的操作；所有改期、取消、退款與審核入口必須對應 06 Command Endpoint</t>
-  </si>
-  <si>
-    <t>階段</t>
-  </si>
-  <si>
-    <t>狀態</t>
-  </si>
-  <si>
-    <t>成熟度</t>
-  </si>
-  <si>
-    <t>下一步</t>
-  </si>
-  <si>
-    <t>00 Project Definition</t>
-  </si>
-  <si>
-    <t>🟢 Done</t>
-  </si>
-  <si>
-    <t>高</t>
-  </si>
-  <si>
-    <t>已完成，維護即可</t>
-  </si>
-  <si>
-    <t>01 PRD</t>
-  </si>
-  <si>
-    <t>PRD 已確認，作為 MVP 需求基準</t>
-  </si>
-  <si>
-    <t>02 Business Rules</t>
-  </si>
-  <si>
-    <t>符號</t>
-  </si>
-  <si>
-    <t>模組</t>
-  </si>
-  <si>
-    <t>Design Baseline，作為 DB / API / Domain / Test 依據</t>
-  </si>
-  <si>
-    <t>03 System Architecture</t>
-  </si>
-  <si>
-    <t>架構基線完成，可支撐 04 Database Design</t>
-  </si>
-  <si>
-    <t>04 Database Design</t>
-  </si>
-  <si>
-    <t>已通過 04-1～04-6 Review Gate，作為 05 輸入基線</t>
-  </si>
-  <si>
-    <t>05 Domain Model</t>
-  </si>
-  <si>
-    <t>優先級</t>
-  </si>
-  <si>
-    <t>Review Gate PASS，可作為 06 API Specification 輸入基線</t>
-  </si>
-  <si>
-    <t>06 API Specification</t>
-  </si>
-  <si>
-    <t>Review Gate PASS；含 Permission / Security、Idempotency、Reschedule、Pricing、Refund</t>
-  </si>
-  <si>
-    <t>07 UI/UX Flow</t>
-  </si>
-  <si>
-    <t>07 Review Gate PASS / Approved Baseline</t>
-  </si>
-  <si>
-    <t>08 Test Strategy</t>
-  </si>
-  <si>
-    <t>08 Review Gate PASS / Approved Baseline；Test Strategy 基線已確認</t>
-  </si>
-  <si>
-    <t>09 Deployment / DevOps</t>
-  </si>
-  <si>
-    <t>09 Review Gate PASS / Approved Baseline；GCP-first Deployment / DevOps 基線已確認</t>
-  </si>
-  <si>
-    <t>說明</t>
-  </si>
-  <si>
-    <t>10 Development</t>
-  </si>
-  <si>
-    <t>單元</t>
-  </si>
-  <si>
-    <t>🟡 Next</t>
-  </si>
-  <si>
-    <t>Ready to Start</t>
-  </si>
-  <si>
-    <t>開始 Repository Bootstrap / MVP Vertical Slice / Spring Boot + React 實作</t>
-  </si>
-  <si>
-    <t>Business Rule</t>
-  </si>
-  <si>
-    <t>11 Future Extensions</t>
-  </si>
-  <si>
     <t>⚪ Not Started</t>
   </si>
   <si>
-    <t>要完成的事情</t>
-  </si>
-  <si>
     <t>非 MVP</t>
   </si>
   <si>
+    <t>Development Ready</t>
+  </si>
+  <si>
     <t>Coupon / Event / Analytics / Court Inventory 依 Roadmap 展開</t>
   </si>
   <si>
-    <t>完成條件</t>
-  </si>
-  <si>
-    <t>DB</t>
-  </si>
-  <si>
-    <t>建議接續順序</t>
-  </si>
-  <si>
-    <t>Domain Model</t>
-  </si>
-  <si>
-    <t>🟢</t>
-  </si>
-  <si>
-    <t>Permission</t>
-  </si>
-  <si>
-    <t>API</t>
-  </si>
-  <si>
-    <t>Test</t>
-  </si>
-  <si>
-    <t>Development Ready</t>
-  </si>
-  <si>
     <t>已收斂，可作為下一階段依據</t>
   </si>
   <si>
+    <t>🟡</t>
+  </si>
+  <si>
+    <t>備註</t>
+  </si>
+  <si>
+    <t>Designing</t>
+  </si>
+  <si>
+    <t>已有方向，但仍需補充規則、流程或細節</t>
+  </si>
+  <si>
+    <t>🔴</t>
+  </si>
+  <si>
+    <t>Gap</t>
+  </si>
+  <si>
     <t>✅ Done</t>
   </si>
   <si>
-    <t>🟡</t>
-  </si>
-  <si>
-    <t>備註</t>
+    <t>目前缺口明顯，開發前必須補齊</t>
+  </si>
+  <si>
+    <t>⚪</t>
+  </si>
+  <si>
+    <t>Not Started</t>
+  </si>
+  <si>
+    <t>會員管理</t>
   </si>
   <si>
     <t>04 Database Design Review</t>
   </si>
   <si>
-    <t>Designing</t>
-  </si>
-  <si>
-    <t>已有方向，但仍需補充規則、流程或細節</t>
-  </si>
-  <si>
-    <t>會員管理</t>
+    <t>尚未開始或尚未討論</t>
   </si>
   <si>
     <t>逐項檢查 Table / FK / Index / Constraint / Check Constraint / Exclusion Constraint</t>
   </si>
   <si>
+    <t>✅</t>
+  </si>
+  <si>
     <t>04-1～04-6 Review Gate PASS</t>
   </si>
   <si>
-    <t>🔴</t>
+    <t>已通過 Requirement / Rule / Domain / DB / Permission / API / Test Gate</t>
   </si>
   <si>
     <t>Done</t>
   </si>
   <si>
-    <t>Gap</t>
-  </si>
-  <si>
-    <t>目前缺口明顯，開發前必須補齊</t>
-  </si>
-  <si>
-    <t>⚪</t>
-  </si>
-  <si>
-    <t>✅</t>
+    <t>❌</t>
+  </si>
+  <si>
+    <t>Not Ready</t>
+  </si>
+  <si>
+    <t>尚未達到可開發條件</t>
   </si>
   <si>
     <t>Business Rules Traceability</t>
   </si>
   <si>
+    <t>把 02 Business Rules 的 BR-xxx 對應到資料表、狀態欄位、Constraint、Audit Log</t>
+  </si>
+  <si>
+    <t>P0 Business Rule 已能找到資料模型支撐</t>
+  </si>
+  <si>
     <t>08 Test Strategy：建立本模組 Contract / Integration / Authorization / State Transition 測試基線</t>
   </si>
   <si>
-    <t>Not Started</t>
-  </si>
-  <si>
-    <t>把 02 Business Rules 的 BR-xxx 對應到資料表、狀態欄位、Constraint、Audit Log</t>
+    <t>Core Domain Boundary Check</t>
+  </si>
+  <si>
+    <t>檢查 Course / Course Session / Enrollment / Payment / Refund / Settlement 邊界</t>
   </si>
   <si>
     <t>多角色與組織權限是核心</t>
   </si>
   <si>
-    <t>尚未開始或尚未討論</t>
+    <t>Aggregate 資料責任清楚，不混用 status</t>
   </si>
   <si>
     <t>球場管理</t>
   </si>
   <si>
-    <t>P0 Business Rule 已能找到資料模型支撐</t>
-  </si>
-  <si>
-    <t>已通過 Requirement / Rule / Domain / DB / Permission / API / Test Gate</t>
+    <t>依 04 Database Design 建立 Aggregate、Entity、Repository Boundary、State Transition、Domain Event</t>
+  </si>
+  <si>
+    <t>05 Review Gate PASS</t>
+  </si>
+  <si>
+    <t>06 API Specification（含 Permission / Security）</t>
+  </si>
+  <si>
+    <t>完成角色與 Organization Scope、Endpoint Contract、Idempotency、Reschedule、Pricing、Refund 與 Security 規格</t>
+  </si>
+  <si>
+    <t>06 Review Gate PASS / Approved Baseline</t>
   </si>
   <si>
     <t>MVP 記錄場地協調，不做即時庫存</t>
   </si>
   <si>
+    <t>已完成 07-UI-UX-Flow.md；Open Enrollment 已確定納入 MVP/P0，且 04 v2.4、05 v1.1、06 v1.1 Backfill Review 全部 PASS</t>
+  </si>
+  <si>
     <t>場地安排 / 球場預約</t>
   </si>
   <si>
-    <t>Core Domain Boundary Check</t>
-  </si>
-  <si>
-    <t>❌</t>
-  </si>
-  <si>
-    <t>Not Ready</t>
-  </si>
-  <si>
-    <t>檢查 Course / Course Session / Enrollment / Payment / Refund / Settlement 邊界</t>
-  </si>
-  <si>
-    <t>尚未達到可開發條件</t>
-  </si>
-  <si>
-    <t>Aggregate 資料責任清楚，不混用 status</t>
+    <t>07 Review Gate PASS / Approved Baseline；Open Enrollment Persistence / Domain / API 已具實作基線，下一階段銜接 08 Test Strategy</t>
+  </si>
+  <si>
+    <t>建立 Contract、State Transition、Authorization、DB Constraint、Concurrency 與 Finance 測試案例</t>
+  </si>
+  <si>
+    <t>08 Review Gate PASS / Approved Baseline</t>
+  </si>
+  <si>
+    <t>建立本機 / Dev 環境、CI/CD、Secret 管理、Flyway 執行與最低監控規範</t>
+  </si>
+  <si>
+    <t>09 Review Gate PASS / Approved Baseline</t>
+  </si>
+  <si>
+    <t>✅ Approved</t>
   </si>
   <si>
     <t>需與課程預約拆清楚</t>
   </si>
   <si>
+    <t>10 Development Review Gate</t>
+  </si>
+  <si>
     <t>教練管理</t>
   </si>
   <si>
-    <t>依 04 Database Design 建立 Aggregate、Entity、Repository Boundary、State Transition、Domain Event</t>
-  </si>
-  <si>
-    <t>05 Review Gate PASS</t>
-  </si>
-  <si>
-    <t>06 API Specification（含 Permission / Security）</t>
-  </si>
-  <si>
-    <t>完成角色與 Organization Scope、Endpoint Contract、Idempotency、Reschedule、Pricing、Refund 與 Security 規格</t>
-  </si>
-  <si>
-    <t>06 Review Gate PASS / Approved Baseline</t>
+    <t>完成 Development Master Plan、Repository 結構、技術版本、Vertical Slice Roadmap、Test / CI / Security / Coding Standards 基線</t>
+  </si>
+  <si>
+    <t>10 Review Gate PASS / Approved Baseline；12 項工程決策全部確認</t>
+  </si>
+  <si>
+    <t>10.1 Repository Bootstrap / Slice 0</t>
+  </si>
+  <si>
+    <t>建立 Monorepo、Backend / Frontend 工程骨架、PostgreSQL 18 local stack、Flyway、Testcontainers、CI skeleton</t>
+  </si>
+  <si>
+    <t>Repository foundation 可 build / test；main 工程骨架完成</t>
+  </si>
+  <si>
+    <t>Slice 1 — Identity / LINE Login / Me / RBAC + Organization Scope</t>
+  </si>
+  <si>
+    <t>完成 Identity Schema、LINE backend verification、JWT、RBAC / Organization Scope、OpenAPI/generated client、LIFF/Admin UX、concurrency、安全與 E2E 測試</t>
   </si>
   <si>
     <t>會影響媒合流程</t>
   </si>
   <si>
-    <t>已完成 07-UI-UX-Flow.md；Open Enrollment 已確定納入 MVP/P0，且 04 v2.4、05 v1.1、06 v1.1 Backfill Review 全部 PASS</t>
+    <t>PR #1 merged；merge commit c1f92549031c025ec7ccfb4c99793300e17efee5；GitHub Actions 全綠；Slice 1 Merge Gate PASS</t>
   </si>
   <si>
     <t>課程需求</t>
   </si>
   <si>
-    <t>07 Review Gate PASS / Approved Baseline；Open Enrollment Persistence / Domain / API 已具實作基線，下一階段銜接 08 Test Strategy</t>
-  </si>
-  <si>
-    <t>建立 Contract、State Transition、Authorization、DB Constraint、Concurrency 與 Finance 測試案例</t>
-  </si>
-  <si>
-    <t>08 Review Gate PASS / Approved Baseline</t>
+    <t>P0</t>
+  </si>
+  <si>
+    <t>Slice 2 Baseline Alignment Backfill 已 PASS；先將最新 02／04／05／06／07／08／10 Approved Baseline 同步到 repository docs/，再實作 Coach Application / single-range Availability / Student Lesson Request、Organization Scope、Idempotency、OpenAPI/client、LIFF/Admin UI 與完整測試</t>
+  </si>
+  <si>
+    <t>Slice 2 Definition of Done 全部 PASS；PR CI 全綠後 Merge main</t>
+  </si>
+  <si>
+    <t>Next — Sync Baseline → Slice 2 Implementation</t>
   </si>
   <si>
     <t>P0 核心；Business Rules 已明確</t>
   </si>
   <si>
-    <t>建立本機 / Dev 環境、CI/CD、Secret 管理、Flyway 執行與最低監控規範</t>
-  </si>
-  <si>
     <t>課程媒合</t>
   </si>
   <si>
-    <t>09 Review Gate PASS / Approved Baseline</t>
-  </si>
-  <si>
-    <t>✅ Approved</t>
-  </si>
-  <si>
-    <t>10 Development Review Gate</t>
-  </si>
-  <si>
-    <t>完成 Development Master Plan、Repository 結構、技術版本、Vertical Slice Roadmap、Test / CI / Security / Coding Standards 基線</t>
-  </si>
-  <si>
-    <t>10 Review Gate PASS / Approved Baseline；12 項工程決策全部確認</t>
-  </si>
-  <si>
     <t>P0 優先</t>
   </si>
   <si>
-    <t>P0</t>
-  </si>
-  <si>
     <t>課程預約</t>
-  </si>
-  <si>
-    <t>建立實際 Git Repository、Backend / Frontend 工程骨架、PostgreSQL 18 local stack、Flyway baseline、Testcontainers、CI skeleton</t>
-  </si>
-  <si>
-    <t>clone 後可 build / test / 啟動 local stack；main CI 綠燈；空白 Vertical Slice 可部署</t>
-  </si>
-  <si>
-    <t>1</t>
   </si>
   <si>
     <t>課程成班</t>
@@ -463,7 +475,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
@@ -518,12 +530,18 @@
     </font>
     <font>
       <b/>
+      <color rgb="FF166534"/>
+      <name val="Carlito"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FF991B1B"/>
       <name val="Carlito"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -562,6 +580,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFDCFCE7"/>
+        <bgColor rgb="FFDCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFEE2E2"/>
         <bgColor rgb="FFFEE2E2"/>
       </patternFill>
@@ -573,7 +597,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -620,10 +644,13 @@
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="7" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf quotePrefix="1" borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="8" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -752,13 +779,13 @@
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
-    <tableStyle count="4" pivot="0" name="狀態定義-style">
+    <tableStyle count="4" pivot="0" name="下一步清單-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
-    <tableStyle count="4" pivot="0" name="下一步清單-style">
+    <tableStyle count="4" pivot="0" name="狀態定義-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -789,7 +816,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J18" displayName="ModuleProgressTable" name="ModuleProgressTable" id="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J18" displayName="ModuleProgressTable" name="ModuleProgressTable" id="1">
   <tableColumns count="10">
     <tableColumn name="模組" id="1"/>
     <tableColumn name="Business Rule" id="2"/>
@@ -807,7 +834,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E11" displayName="NextStepsTable" name="NextStepsTable" id="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E13" displayName="NextStepsTable" name="NextStepsTable" id="3">
   <tableColumns count="5">
     <tableColumn name="優先級" id="1"/>
     <tableColumn name="單元" id="2"/>
@@ -820,7 +847,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C7" displayName="StatusLegendTable" name="StatusLegendTable" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C7" displayName="StatusLegendTable" name="StatusLegendTable" id="2">
   <tableColumns count="3">
     <tableColumn name="符號" id="1"/>
     <tableColumn name="狀態" id="2"/>
@@ -1094,98 +1121,86 @@
       <c r="C5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>9</v>
-      </c>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>9</v>
-      </c>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>9</v>
-      </c>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="C10" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="D10" s="9" t="s">
         <v>18</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="C11" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="D11" s="6" t="s">
         <v>22</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>22</v>
-      </c>
       <c r="D12" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B13" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>29</v>
@@ -1196,10 +1211,10 @@
         <v>30</v>
       </c>
       <c r="B14" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>31</v>
@@ -1210,10 +1225,10 @@
         <v>32</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>33</v>
@@ -1224,10 +1239,10 @@
         <v>34</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>36</v>
@@ -1235,86 +1250,86 @@
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="6" t="s">
-        <v>22</v>
-      </c>
       <c r="D17" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B18" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="6" t="s">
-        <v>22</v>
-      </c>
       <c r="D18" s="6" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B19" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="6" t="s">
-        <v>22</v>
-      </c>
       <c r="D19" s="6" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B20" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="6" t="s">
-        <v>22</v>
-      </c>
       <c r="D20" s="6" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="6" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>49</v>
+        <v>7</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="6" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1"/>
@@ -2349,34 +2364,34 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="E1" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="H1" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="F1" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="H1" s="10" t="s">
-        <v>65</v>
-      </c>
       <c r="I1" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
@@ -2397,543 +2412,543 @@
     </row>
     <row r="2">
       <c r="A2" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="G2" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="B2" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="D2" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="F2" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="G2" s="13" t="s">
-        <v>80</v>
-      </c>
       <c r="H2" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I2" s="13" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="J2" s="13" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I8" s="13" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="J8" s="13" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="J11" s="13" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="J14" s="13" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="G15" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="H15" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="I15" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="J15" s="13" t="s">
         <v>140</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="G15" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="H15" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="I15" s="13" t="s">
-        <v>135</v>
-      </c>
-      <c r="J15" s="13" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="J16" s="13" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="J17" s="13" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
+        <v>79</v>
+      </c>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -4073,19 +4088,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -4111,171 +4126,205 @@
     </row>
     <row r="2">
       <c r="A2" s="13" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B3" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="E3" s="13" t="s">
         <v>82</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B4" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="C4" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>98</v>
-      </c>
       <c r="E4" s="13" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>34</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11" ht="43.5" customHeight="1">
+      <c r="A11" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="D11" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="E11" s="16" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="12" ht="43.5" customHeight="1">
+      <c r="A12" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C12" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="D10" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>77</v>
+      <c r="D12" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>82</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="14" t="s">
+    <row r="13" ht="43.5" customHeight="1">
+      <c r="A13" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D13" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E13" s="16" t="s">
         <v>125</v>
       </c>
     </row>
@@ -5300,13 +5349,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -5334,68 +5383,68 @@
     </row>
     <row r="2">
       <c r="A2" s="12" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>7</v>
+        <v>59</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>68</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>